<commit_message>
Corte MPOO: una P03 mas, en equipo declarado
</commit_message>
<xml_diff>
--- a/calificaciones/P00-P03-corte-12sep.xlsx
+++ b/calificaciones/P00-P03-corte-12sep.xlsx
@@ -14,8 +14,7 @@
     <sheet name="323065115" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="319112375" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="322287123" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="426058988" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="323272733" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="323272733" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1650,9 +1649,9 @@
           <t>10</t>
         </is>
       </c>
-      <c r="E33" s="11" t="inlineStr">
-        <is>
-          <t>PC</t>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
@@ -1662,7 +1661,7 @@
       </c>
       <c r="G33" s="10" t="inlineStr">
         <is>
-          <t>Solo subiste el Laboratorio.class: falta el Laboratorio.java y el documento con tu captura y tu analisis, que es la mayor parte de la practica. Ver tu hoja.</t>
+          <t>Completa, en equipo declarado. Para la proxima: sube tambien tu .java y tu documento en tu carpeta, aunque el trabajo sea de equipo.</t>
         </is>
       </c>
     </row>
@@ -1771,14 +1770,14 @@
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>P03:  correctas 14   ·   pendientes de correccion 1   ·   no presentadas 14</t>
+          <t>P03:  correctas 15   ·   pendientes de correccion 0   ·   no presentadas 14</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>Las cuatro completas y correctas: 13 de 29     ·     Sin ninguna entrega: 2 de 29</t>
+          <t>Las cuatro completas y correctas: 14 de 29     ·     Sin ninguna entrega: 2 de 29</t>
         </is>
       </c>
     </row>
@@ -2602,144 +2601,6 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Correccion · 426058988</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 426058988   ·   Por corregir: P03</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="13" t="inlineStr">
-        <is>
-          <t>P00: 10    P01: 10    P02: 10    P03: PC</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="17" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="56" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>Solo subiste el Laboratorio.class. Falta el Laboratorio.java con tu bloque 7 y falta el documento con la captura de tu tabla final y tu analisis, que juntos son la mayor parte de la calificacion.</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>Sube tu Laboratorio.java y tu documento. Si ya corriste el programa, la tabla final tambien quedo en mis-resultados.txt, en la misma carpeta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>Tu profesor va a revisar contigo esta entrega antes de calificarla.</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Acercate con el en la proxima sesion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="20" t="inlineStr">
-        <is>
-          <t>git fetch origin</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="20" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="20" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="20" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="20" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/pNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="20" t="inlineStr">
-        <is>
-          <t>git commit -m "PNN: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="20" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="21" t="inlineStr">
-        <is>
-          <t>No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="16" t="inlineStr">
-        <is>
           <t>Correccion · 323272733</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Corte MPOO: una P03 queda incompleta
</commit_message>
<xml_diff>
--- a/calificaciones/P00-P03-corte-12sep.xlsx
+++ b/calificaciones/P00-P03-corte-12sep.xlsx
@@ -14,7 +14,8 @@
     <sheet name="323065115" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="319112375" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="322287123" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="323272733" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="426058988" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="323272733" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1649,9 +1650,9 @@
           <t>10</t>
         </is>
       </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>10</t>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>PC</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
@@ -1661,7 +1662,7 @@
       </c>
       <c r="G33" s="10" t="inlineStr">
         <is>
-          <t>Completa, en equipo declarado. Para la proxima: sube tambien tu .java y tu documento en tu carpeta, aunque el trabajo sea de equipo.</t>
+          <t>Incompleta: en tu carpeta solo esta el Laboratorio.class. Aunque el trabajo sea de equipo, cada quien sube su .java y su documento con la captura y el analisis. Ver tu hoja.</t>
         </is>
       </c>
     </row>
@@ -1770,14 +1771,14 @@
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>P03:  correctas 15   ·   pendientes de correccion 0   ·   no presentadas 14</t>
+          <t>P03:  correctas 14   ·   pendientes de correccion 1   ·   no presentadas 14</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>Las cuatro completas y correctas: 14 de 29     ·     Sin ninguna entrega: 2 de 29</t>
+          <t>Las cuatro completas y correctas: 13 de 29     ·     Sin ninguna entrega: 2 de 29</t>
         </is>
       </c>
     </row>
@@ -2601,6 +2602,144 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
+          <t>Correccion · 426058988</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta: 426058988   ·   Por corregir: P03</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>P00: 10    P01: 10    P02: 10    P03: PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Que hay que corregir</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Como se corrige</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="56" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>En tu carpeta solo esta el Laboratorio.class. Falta el Laboratorio.java con tu bloque 7, y falta el documento con la captura de la tabla final y tu analisis: entre los dos son la mayor parte de la calificacion.</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Sube los dos a entregas/tu_apellido_nombre/p03/. Si ya corriste el programa, la tabla tambien quedo guardada en mis-resultados.txt, en esa misma carpeta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>El trabajo en equipo esta permitido, pero la entrega es individual.</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Aunque lo hayan resuelto juntas, cada quien sube sus archivos en su propia carpeta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>git fetch origin</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>(corrige tus archivos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>git add entregas/tu_apellido_nombre/pNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>git commit -m "PNN: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>No abras pull request: el push ES la entrega.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
           <t>Correccion · 323272733</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Corte MPOO: quedan pendientes los que aparecen como equipo pero sin entrega en su carpeta
</commit_message>
<xml_diff>
--- a/calificaciones/P00-P03-corte-12sep.xlsx
+++ b/calificaciones/P00-P03-corte-12sep.xlsx
@@ -8,14 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="Matriz" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="322098930" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="323290577" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="322179684" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="323065115" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="319112375" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="322287123" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="426058988" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="323272733" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="323297291" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="322098930" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="323290577" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="322179684" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="323065115" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="319112375" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="322287123" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="322153686" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="426058988" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="322095458" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="323272733" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -725,9 +728,9 @@
           <t>10</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>NP</t>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>PC</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
@@ -737,7 +740,7 @@
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>Completa hasta P02. Tu P03 no esta subida en tu rama, aunque apareces como equipo en el documento de tu companero.</t>
+          <t>Tu P03 no esta en tu carpeta, aunque apareces como equipo en el documento de tu companero. Aunque lo hayan hecho juntos, cada quien sube sus archivos. Ver tu hoja.</t>
         </is>
       </c>
     </row>
@@ -1576,9 +1579,9 @@
           <t>10</t>
         </is>
       </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>NP</t>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>PC</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
@@ -1588,7 +1591,7 @@
       </c>
       <c r="G31" s="10" t="inlineStr">
         <is>
-          <t>Tu P03 no esta subida en tu rama, aunque apareces como equipo en el documento de tu companero.</t>
+          <t>Tu P03 no esta en tu carpeta, aunque apareces como equipo en el documento de tu companero. Aunque lo hayan hecho juntos, cada quien sube sus archivos. Ver tu hoja.</t>
         </is>
       </c>
     </row>
@@ -1687,9 +1690,9 @@
           <t>10</t>
         </is>
       </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>NP</t>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>PC</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
@@ -1699,7 +1702,7 @@
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
-          <t>Completa hasta la P02. Falta la P03.</t>
+          <t>Tu P03 no esta en tu carpeta, aunque apareces como equipo en el documento de tu companero. Aunque lo hayan hecho juntos, cada quien sube sus archivos. Ver tu hoja.</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1774,7 @@
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>P03:  correctas 14   ·   pendientes de correccion 1   ·   no presentadas 14</t>
+          <t>P03:  correctas 14   ·   pendientes de correccion 4   ·   no presentadas 11</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1797,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1810,21 +1813,21 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Correccion · 322098930</t>
+          <t>Correccion · 426058988</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 322098930   ·   Por corregir: P03</t>
+          <t>Cuenta: 426058988   ·   Por corregir: P03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: 10    P01: 10    P02: 10    P03: 9</t>
+          <t>P00: 10    P01: 10    P02: 10    P03: PC</t>
         </is>
       </c>
     </row>
@@ -1840,27 +1843,27 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1">
+    <row r="6" ht="56" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>No entregaste el Laboratorio.java del curso. Subiste un programa propio que tiene los 36 resultados escritos a mano en un arreglo: no calcula nada, solo los imprime.</t>
+          <t>En tu carpeta solo esta el Laboratorio.class. Falta el Laboratorio.java con tu bloque 7, y falta el documento con la captura de la tabla final y tu analisis: entre los dos son la mayor parte de la calificacion.</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Baja el Laboratorio.java de guias-laboratorios/Lab-03/, correlo, contesta las 36 y sube ESE archivo con tu bloque 7 escrito.</t>
+          <t>Sube los dos a entregas/tu_apellido_nombre/p03/. Si ya corriste el programa, la tabla tambien quedo guardada en mis-resultados.txt, en esa misma carpeta.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>Por lo mismo, no tienes bloque 7.</t>
+          <t>El trabajo en equipo esta permitido, pero la entrega es individual.</t>
         </is>
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>Son las 5 lineas del final: descomentalas y completalas. Tu documento y tu analisis si estan bien, esos no le muevas.</t>
+          <t>Aunque lo hayan resuelto juntas, cada quien sube sus archivos en su propia carpeta.</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1935,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1948,21 +1951,21 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Correccion · 323290577</t>
+          <t>Correccion · 322095458</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 323290577   ·   Por corregir: P02</t>
+          <t>Cuenta: 322095458   ·   Por corregir: P03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: 10    P01: 10    P02: PC    P03: NP</t>
+          <t>P00: 10    P01: 10    P02: 10    P03: PC</t>
         </is>
       </c>
     </row>
@@ -1981,12 +1984,12 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>Tu P02 no compila: PruebaPunto3 y PruebaPunto4 crean el objeto con new Punto(5,8), pero tu clase Punto no tiene constructor con parametros.</t>
+          <t>Tu P03 no esta en tu carpeta. Apareces como equipo en el documento de tu companero, pero ahi no hay archivos tuyos.</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>O le agregas a Punto el constructor Punto(int x, int y), o cambias esas pruebas para que usen la clase que si lo tiene.</t>
+          <t>Sube en entregas/tu_apellido_nombre/p03/ tu Laboratorio.java con el bloque 7, tu .class y el documento. Puede ser el mismo trabajo del equipo.</t>
         </is>
       </c>
     </row>
@@ -2048,6 +2051,408 @@
     </row>
     <row r="16">
       <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>No abras pull request: el push ES la entrega.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Correccion · 323272733</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta: 323272733   ·   Por corregir: P03</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>P00: 10    P01: 10    P02: 10    P03: 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Que hay que corregir</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Como se corrige</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>No entregaste el Laboratorio.java de la practica: subiste un programa distinto, con los 36 resultados escritos a mano en un arreglo, que no calcula nada.</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Baja el Laboratorio.java de guias-laboratorios/Lab-03/, escribe ahi tu bloque 7 y sube ESE archivo. Tu documento y tu analisis estan muy bien, esos no le muevas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Por lo mismo, tu bloque 7 no existe (0 de 5).</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Son las cinco lineas del final: descomentalas y completalas con operaciones de verdad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>git fetch origin</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>(corrige tus archivos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>git add entregas/tu_apellido_nombre/pNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>git commit -m "PNN: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>No abras pull request: el push ES la entrega.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Correccion · 323297291</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta: 323297291   ·   Por corregir: P03</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>P00: 10    P01: 10    P02: 10    P03: PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Que hay que corregir</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Como se corrige</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="56" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Tu P03 no esta en tu carpeta. Apareces como equipo en el documento de tu companero, pero ahi no hay archivos tuyos.</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Sube en entregas/tu_apellido_nombre/p03/ tu Laboratorio.java con el bloque 7, tu .class y el documento. Puede ser el mismo trabajo del equipo: lo que falta es que este tambien en tu carpeta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>git fetch origin</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>(corrige tus archivos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>git add entregas/tu_apellido_nombre/pNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>git commit -m "PNN: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>No abras pull request: el push ES la entrega.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Correccion · 322098930</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta: 322098930   ·   Por corregir: P03</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>P00: 10    P01: 10    P02: 10    P03: 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Que hay que corregir</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Como se corrige</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>No entregaste el Laboratorio.java del curso. Subiste un programa propio que tiene los 36 resultados escritos a mano en un arreglo: no calcula nada, solo los imprime.</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Baja el Laboratorio.java de guias-laboratorios/Lab-03/, correlo, contesta las 36 y sube ESE archivo con tu bloque 7 escrito.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Por lo mismo, no tienes bloque 7.</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Son las 5 lineas del final: descomentalas y completalas. Tu documento y tu analisis si estan bien, esos no le muevas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>git fetch origin</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>(corrige tus archivos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>git add entregas/tu_apellido_nombre/pNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>git commit -m "PNN: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2074,21 +2479,21 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Correccion · 322179684</t>
+          <t>Correccion · 323290577</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 322179684   ·   Por corregir: P02</t>
+          <t>Cuenta: 323290577   ·   Por corregir: P02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: 10    P01: 10    P02: 10    P03: 10</t>
+          <t>P00: 10    P01: 10    P02: PC    P03: NP</t>
         </is>
       </c>
     </row>
@@ -2107,12 +2512,12 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>Tu variante de constructores ya quedo: le agregamos el constructor que faltaba desde tu rama vieja y ya compila.</t>
+          <t>Tu P02 no compila: PruebaPunto3 y PruebaPunto4 crean el objeto con new Punto(5,8), pero tu clase Punto no tiene constructor con parametros.</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada aqui. Solo trabaja de aqui en adelante en tu rama entregas_, no en las viejas.</t>
+          <t>O le agregas a Punto el constructor Punto(int x, int y), o cambias esas pruebas para que usen la clase que si lo tiene.</t>
         </is>
       </c>
     </row>
@@ -2200,21 +2605,21 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Correccion · 323065115</t>
+          <t>Correccion · 322179684</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 323065115   ·   Por corregir: P03 · solo te falta el bloque 7</t>
+          <t>Cuenta: 322179684   ·   Por corregir: P02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: 10    P01: 10    P02: 9    P03: 9</t>
+          <t>P00: 10    P01: 10    P02: 10    P03: 10</t>
         </is>
       </c>
     </row>
@@ -2233,12 +2638,12 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>Te falta todo el bloque 7: las cinco lineas siguen comentadas, tal como venia el archivo.</t>
+          <t>Tu variante de constructores ya quedo: le agregamos el constructor que faltaba desde tu rama vieja y ya compila.</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Descomentalas y completalas. Cada una tiene que ser una operacion de verdad, con un comentario diciendo que operador usaste.</t>
+          <t>No tienes que hacer nada aqui. Solo trabaja de aqui en adelante en tu rama entregas_, no en las viejas.</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -2326,21 +2731,21 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Correccion · 319112375</t>
+          <t>Correccion · 323065115</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 319112375   ·   Por corregir: P03</t>
+          <t>Cuenta: 323065115   ·   Por corregir: P03 · solo te falta el bloque 7</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: 10    P01: NP    P02: NP    P03: 8</t>
+          <t>P00: 10    P01: 10    P02: 9    P03: 9</t>
         </is>
       </c>
     </row>
@@ -2359,85 +2764,73 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>Te falta todo el bloque 7: las cinco lineas siguen comentadas. Tu Laboratorio.java esta identico al que se te dio.</t>
+          <t>Te falta todo el bloque 7: las cinco lineas siguen comentadas, tal como venia el archivo.</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Descomentalas y completalas, y vuelve a subir el archivo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>No entregaste el documento con tu analisis, que es la mitad de la calificacion.</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Corre el programa, toma captura de la tabla final y escribe por que fallaste las 4 que fallaste. Acertaste 32 de 36: te falta poco.</t>
+          <t>Descomentalas y completalas. Cada una tiene que ser una operacion de verdad, con un comentario diciendo que operador usaste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>git fetch origin</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t>git fetch origin</t>
+          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="inlineStr">
         <is>
-          <t>git checkout TU-RAMA</t>
+          <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>git pull origin main</t>
+          <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="inlineStr">
         <is>
-          <t>(corrige tus archivos)</t>
+          <t>git add entregas/tu_apellido_nombre/pNN</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>git add entregas/tu_apellido_nombre/pNN</t>
+          <t>git commit -m "PNN: correccion"</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="inlineStr">
         <is>
-          <t>git commit -m "PNN: correccion"</t>
+          <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2464,21 +2857,21 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Correccion · 322287123</t>
+          <t>Correccion · 319112375</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 322287123   ·   Por corregir: P03</t>
+          <t>Cuenta: 319112375   ·   Por corregir: P03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: 10    P01: 10    P02: 10    P03: 9</t>
+          <t>P00: 10    P01: NP    P02: NP    P03: 8</t>
         </is>
       </c>
     </row>
@@ -2497,24 +2890,24 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>Falta la captura de la TABLA FINAL, la que dice 'TU TABLA FINAL · ESTA ES LA CAPTURA QUE TIENES QUE ENTREGAR'. Tu PDF termina en el bloque 6.</t>
+          <t>Te falta todo el bloque 7: las cinco lineas siguen comentadas. Tu Laboratorio.java esta identico al que se te dio.</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Corre el programa hasta el final y toma captura de esa tabla; tambien quedo guardada en mis-resultados.txt.</t>
+          <t>Descomentalas y completalas, y vuelve a subir el archivo.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>Tu analisis va por temas y fallaste 13 predicciones.</t>
+          <t>No entregaste el documento con tu analisis, que es la mitad de la calificacion.</t>
         </is>
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>Lo que se califica es explicar CADA falla: que creias tu y que hace en realidad Java. Tu bloque 7 quedo muy bien, ese no le muevas.</t>
+          <t>Corre el programa, toma captura de la tabla final y escribe por que fallaste las 4 que fallaste. Acertaste 32 de 36: te falta poco.</t>
         </is>
       </c>
     </row>
@@ -2602,21 +2995,21 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Correccion · 426058988</t>
+          <t>Correccion · 322287123</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 426058988   ·   Por corregir: P03</t>
+          <t>Cuenta: 322287123   ·   Por corregir: P03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: 10    P01: 10    P02: 10    P03: PC</t>
+          <t>P00: 10    P01: 10    P02: 10    P03: 9</t>
         </is>
       </c>
     </row>
@@ -2632,27 +3025,27 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="56" customHeight="1">
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>En tu carpeta solo esta el Laboratorio.class. Falta el Laboratorio.java con tu bloque 7, y falta el documento con la captura de la tabla final y tu analisis: entre los dos son la mayor parte de la calificacion.</t>
+          <t>Falta la captura de la TABLA FINAL, la que dice 'TU TABLA FINAL · ESTA ES LA CAPTURA QUE TIENES QUE ENTREGAR'. Tu PDF termina en el bloque 6.</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Sube los dos a entregas/tu_apellido_nombre/p03/. Si ya corriste el programa, la tabla tambien quedo guardada en mis-resultados.txt, en esa misma carpeta.</t>
+          <t>Corre el programa hasta el final y toma captura de esa tabla; tambien quedo guardada en mis-resultados.txt.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>El trabajo en equipo esta permitido, pero la entrega es individual.</t>
+          <t>Tu analisis va por temas y fallaste 13 predicciones.</t>
         </is>
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>Aunque lo hayan resuelto juntas, cada quien sube sus archivos en su propia carpeta.</t>
+          <t>Lo que se califica es explicar CADA falla: que creias tu y que hace en realidad Java. Tu bloque 7 quedo muy bien, ese no le muevas.</t>
         </is>
       </c>
     </row>
@@ -2730,7 +3123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -2740,21 +3133,21 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Correccion · 323272733</t>
+          <t>Correccion · 322153686</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 323272733   ·   Por corregir: P03</t>
+          <t>Cuenta: 322153686   ·   Por corregir: P03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: 10    P01: 10    P02: 10    P03: 9</t>
+          <t>P00: 10    P01: 9    P02: 10    P03: PC</t>
         </is>
       </c>
     </row>
@@ -2770,88 +3163,76 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1">
+    <row r="6" ht="56" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>No entregaste el Laboratorio.java de la practica: subiste un programa distinto, con los 36 resultados escritos a mano en un arreglo, que no calcula nada.</t>
+          <t>Tu P03 no esta en tu carpeta. Apareces como equipo en el documento de tu companero, y sus capturas muestran que corrieron desde tu carpeta, pero ahi no quedaron los archivos.</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Baja el Laboratorio.java de guias-laboratorios/Lab-03/, escribe ahi tu bloque 7 y sube ESE archivo. Tu documento y tu analisis estan muy bien, esos no le muevas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>Por lo mismo, tu bloque 7 no existe (0 de 5).</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Son las cinco lineas del final: descomentalas y completalas con operaciones de verdad.</t>
+          <t>Sube en entregas/tu_apellido_nombre/p03/ tu Laboratorio.java con el bloque 7, tu .class y el documento. Puede ser el mismo trabajo del equipo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>git fetch origin</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t>git fetch origin</t>
+          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="inlineStr">
         <is>
-          <t>git checkout TU-RAMA</t>
+          <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>git pull origin main</t>
+          <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="inlineStr">
         <is>
-          <t>(corrige tus archivos)</t>
+          <t>git add entregas/tu_apellido_nombre/pNN</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>git add entregas/tu_apellido_nombre/pNN</t>
+          <t>git commit -m "PNN: correccion"</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="inlineStr">
         <is>
-          <t>git commit -m "PNN: correccion"</t>
+          <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>No abras pull request: el push ES la entrega.</t>
         </is>

</xml_diff>